<commit_message>
Fix spell and example
</commit_message>
<xml_diff>
--- a/public/example/main.xlsx
+++ b/public/example/main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\github\jonaskello\backcel\public\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBFEBACC-DFA3-48EF-B107-2515E3C80EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1422E242-0151-43AC-B34B-F6FBDDBBE91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="7" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="103">
   <si>
     <t>ID</t>
   </si>
@@ -346,6 +346,9 @@
   </si>
   <si>
     <t>__rb_check</t>
+  </si>
+  <si>
+    <t>_portfolios</t>
   </si>
 </sst>
 </file>
@@ -766,7 +769,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B8" t="s">
         <v>79</v>

</xml_diff>